<commit_message>
Ignacio's changes on cluster plots
</commit_message>
<xml_diff>
--- a/MASTER/cluster_plots_loadings/agg/pca_results_agg.xlsx
+++ b/MASTER/cluster_plots_loadings/agg/pca_results_agg.xlsx
@@ -1025,20 +1025,20 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No oil, minerals</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.74983281537278</v>
+        <v>-3.739555103476817</v>
       </c>
       <c r="C2" t="n">
-        <v>1.090887736438717</v>
+        <v>3.470858045496856</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No oil, no minerals</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1051,7 +1051,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Oil, no minerals</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1064,14 +1064,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Oil, some minerals</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>-3.739555103476817</v>
+        <v>4.74983281537278</v>
       </c>
       <c r="C5" t="n">
-        <v>3.470858045496856</v>
+        <v>1.090887736438717</v>
       </c>
     </row>
   </sheetData>
@@ -1108,20 +1108,20 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No oil, minerals</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2.070071043800124</v>
+        <v>0.8692227322787303</v>
       </c>
       <c r="C2" t="n">
-        <v>2.144158416364655</v>
+        <v>1.7047369014996</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No oil, no minerals</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1134,7 +1134,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Oil, no minerals</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1147,14 +1147,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Oil, some minerals</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8692227322787303</v>
+        <v>2.070071043800124</v>
       </c>
       <c r="C5" t="n">
-        <v>1.7047369014996</v>
+        <v>2.144158416364655</v>
       </c>
     </row>
   </sheetData>
@@ -1186,17 +1186,17 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No oil, minerals</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No oil, no minerals</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1206,7 +1206,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Oil, no minerals</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1216,11 +1216,11 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Oil, some minerals</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1257,7 +1257,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No oil, minerals</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>4.74983281537278</v>
+        <v>-3.739555103476817</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No oil, no minerals</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Oil, no minerals</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Oil, some minerals</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1311,13 +1311,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>-3.739555103476817</v>
+        <v>4.74983281537278</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>No oil, minerals</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.090887736438717</v>
+        <v>3.470858045496856</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No oil, no minerals</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1347,7 +1347,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Oil, no minerals</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1362,7 +1362,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Oil, some minerals</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3.470858045496856</v>
+        <v>1.090887736438717</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Merge branch 'main' of https://github.com/AyaanTigdikar/Capstone"
This reverts commit 41a62260f101124089c001af94f5e5d821f266f9, reversing
changes made to a25f3f841b4776e4e71c4fc094b6c6e142a18180.
</commit_message>
<xml_diff>
--- a/MASTER/cluster_plots_loadings/agg/pca_results_agg.xlsx
+++ b/MASTER/cluster_plots_loadings/agg/pca_results_agg.xlsx
@@ -1025,20 +1025,20 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>No oil, minerals</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-3.739555103476817</v>
+        <v>4.74983281537278</v>
       </c>
       <c r="C2" t="n">
-        <v>3.470858045496856</v>
+        <v>1.090887736438717</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>No oil, no minerals</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1051,7 +1051,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Oil, no minerals</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1064,14 +1064,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Oil, some minerals</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4.74983281537278</v>
+        <v>-3.739555103476817</v>
       </c>
       <c r="C5" t="n">
-        <v>1.090887736438717</v>
+        <v>3.470858045496856</v>
       </c>
     </row>
   </sheetData>
@@ -1108,20 +1108,20 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>No oil, minerals</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.8692227322787303</v>
+        <v>2.070071043800124</v>
       </c>
       <c r="C2" t="n">
-        <v>1.7047369014996</v>
+        <v>2.144158416364655</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>No oil, no minerals</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1134,7 +1134,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Oil, no minerals</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1147,14 +1147,14 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Oil, some minerals</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2.070071043800124</v>
+        <v>0.8692227322787303</v>
       </c>
       <c r="C5" t="n">
-        <v>2.144158416364655</v>
+        <v>1.7047369014996</v>
       </c>
     </row>
   </sheetData>
@@ -1186,17 +1186,17 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>No oil, minerals</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>No oil, no minerals</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -1206,7 +1206,7 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Oil, no minerals</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -1216,11 +1216,11 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Oil, some minerals</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>15</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1257,7 +1257,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No oil, minerals</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-3.739555103476817</v>
+        <v>4.74983281537278</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>No oil, no minerals</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1287,7 +1287,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oil, no minerals</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1302,7 +1302,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Oil, some minerals</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1311,13 +1311,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.74983281537278</v>
+        <v>-3.739555103476817</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>No oil, minerals</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1326,13 +1326,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3.470858045496856</v>
+        <v>1.090887736438717</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>No oil, no minerals</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1347,7 +1347,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oil, no minerals</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1362,7 +1362,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Oil, some minerals</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1371,7 +1371,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.090887736438717</v>
+        <v>3.470858045496856</v>
       </c>
     </row>
   </sheetData>

</xml_diff>